<commit_message>
Ajustes de modelo bot
</commit_message>
<xml_diff>
--- a/Rodovias/modelos_rodovias/doutor_manoel_hyppolito_rego_km_83_caraguatatuba_sp_rf_regimes/predicoes_teste.xlsx
+++ b/Rodovias/modelos_rodovias/doutor_manoel_hyppolito_rego_km_83_caraguatatuba_sp_rf_regimes/predicoes_teste.xlsx
@@ -969,7 +969,7 @@
         <v>8964</v>
       </c>
       <c r="BM2" t="n">
-        <v>0.3131644635617932</v>
+        <v>0.3131644635617931</v>
       </c>
       <c r="BN2" t="n">
         <v>0</v>
@@ -1632,7 +1632,7 @@
         <v>5229</v>
       </c>
       <c r="BM5" t="n">
-        <v>0.741925576438067</v>
+        <v>0.7419255764380671</v>
       </c>
       <c r="BN5" t="n">
         <v>1</v>
@@ -1853,7 +1853,7 @@
         <v>6600</v>
       </c>
       <c r="BM6" t="n">
-        <v>0.6960697166453838</v>
+        <v>0.6960697166453839</v>
       </c>
       <c r="BN6" t="n">
         <v>1</v>
@@ -2074,7 +2074,7 @@
         <v>9240</v>
       </c>
       <c r="BM7" t="n">
-        <v>0.3039589674521105</v>
+        <v>0.3039589674521104</v>
       </c>
       <c r="BN7" t="n">
         <v>0</v>
@@ -2516,7 +2516,7 @@
         <v>5720</v>
       </c>
       <c r="BM9" t="n">
-        <v>0.6580230673779627</v>
+        <v>0.6580230673779626</v>
       </c>
       <c r="BN9" t="n">
         <v>1</v>
@@ -2737,7 +2737,7 @@
         <v>4048</v>
       </c>
       <c r="BM10" t="n">
-        <v>0.7790208964928838</v>
+        <v>0.7790208964928839</v>
       </c>
       <c r="BN10" t="n">
         <v>1</v>
@@ -3400,7 +3400,7 @@
         <v>8008</v>
       </c>
       <c r="BM13" t="n">
-        <v>0.236507005539043</v>
+        <v>0.2365070055390429</v>
       </c>
       <c r="BN13" t="n">
         <v>0</v>
@@ -4063,7 +4063,7 @@
         <v>8439</v>
       </c>
       <c r="BM16" t="n">
-        <v>0.2015646465688333</v>
+        <v>0.2015646465688334</v>
       </c>
       <c r="BN16" t="n">
         <v>0</v>
@@ -4284,7 +4284,7 @@
         <v>5394</v>
       </c>
       <c r="BM17" t="n">
-        <v>0.4766871611733952</v>
+        <v>0.4766871611733953</v>
       </c>
       <c r="BN17" t="n">
         <v>0</v>
@@ -9367,7 +9367,7 @@
         <v>5280</v>
       </c>
       <c r="BM40" t="n">
-        <v>0.3870467616926192</v>
+        <v>0.3870467616926194</v>
       </c>
       <c r="BN40" t="n">
         <v>0</v>
@@ -9588,7 +9588,7 @@
         <v>3680</v>
       </c>
       <c r="BM41" t="n">
-        <v>0.533522408254133</v>
+        <v>0.5335224082541328</v>
       </c>
       <c r="BN41" t="n">
         <v>1</v>
@@ -10472,7 +10472,7 @@
         <v>4400</v>
       </c>
       <c r="BM45" t="n">
-        <v>0.688393767930691</v>
+        <v>0.6883937679306908</v>
       </c>
       <c r="BN45" t="n">
         <v>1</v>
@@ -11798,7 +11798,7 @@
         <v>4800</v>
       </c>
       <c r="BM51" t="n">
-        <v>0.5706437627020652</v>
+        <v>0.5706437627020653</v>
       </c>
       <c r="BN51" t="n">
         <v>1</v>
@@ -14892,7 +14892,7 @@
         <v>4071</v>
       </c>
       <c r="BM65" t="n">
-        <v>0.6275138144570117</v>
+        <v>0.6275138144570116</v>
       </c>
       <c r="BN65" t="n">
         <v>1</v>
@@ -15776,7 +15776,7 @@
         <v>2415</v>
       </c>
       <c r="BM69" t="n">
-        <v>0.6619566824516027</v>
+        <v>0.6619566824516026</v>
       </c>
       <c r="BN69" t="n">
         <v>1</v>
@@ -17544,7 +17544,7 @@
         <v>8056</v>
       </c>
       <c r="BM77" t="n">
-        <v>0.1424768961083157</v>
+        <v>0.1424768961083158</v>
       </c>
       <c r="BN77" t="n">
         <v>0</v>
@@ -19091,7 +19091,7 @@
         <v>10320</v>
       </c>
       <c r="BM84" t="n">
-        <v>0.2712126107034818</v>
+        <v>0.2712126107034817</v>
       </c>
       <c r="BN84" t="n">
         <v>0</v>
@@ -19312,7 +19312,7 @@
         <v>7826</v>
       </c>
       <c r="BM85" t="n">
-        <v>0.4567305325607038</v>
+        <v>0.4567305325607037</v>
       </c>
       <c r="BN85" t="n">
         <v>0</v>
@@ -24395,7 +24395,7 @@
         <v>7912</v>
       </c>
       <c r="BM108" t="n">
-        <v>0.3306719781104871</v>
+        <v>0.3306719781104872</v>
       </c>
       <c r="BN108" t="n">
         <v>0</v>
@@ -25058,7 +25058,7 @@
         <v>3990</v>
       </c>
       <c r="BM111" t="n">
-        <v>0.5965592438426692</v>
+        <v>0.5965592438426691</v>
       </c>
       <c r="BN111" t="n">
         <v>1</v>
@@ -25279,7 +25279,7 @@
         <v>5035</v>
       </c>
       <c r="BM112" t="n">
-        <v>0.6195030478644344</v>
+        <v>0.6195030478644346</v>
       </c>
       <c r="BN112" t="n">
         <v>1</v>
@@ -26605,7 +26605,7 @@
         <v>7220</v>
       </c>
       <c r="BM118" t="n">
-        <v>0.3216289091596432</v>
+        <v>0.3216289091596433</v>
       </c>
       <c r="BN118" t="n">
         <v>0</v>
@@ -27710,7 +27710,7 @@
         <v>7695</v>
       </c>
       <c r="BM123" t="n">
-        <v>0.2960635545210545</v>
+        <v>0.2960635545210544</v>
       </c>
       <c r="BN123" t="n">
         <v>0</v>
@@ -28152,7 +28152,7 @@
         <v>1785</v>
       </c>
       <c r="BM125" t="n">
-        <v>0.7575348126222533</v>
+        <v>0.7575348126222534</v>
       </c>
       <c r="BN125" t="n">
         <v>1</v>
@@ -28373,7 +28373,7 @@
         <v>2125</v>
       </c>
       <c r="BM126" t="n">
-        <v>0.7214961089453551</v>
+        <v>0.721496108945355</v>
       </c>
       <c r="BN126" t="n">
         <v>1</v>
@@ -29478,7 +29478,7 @@
         <v>2349</v>
       </c>
       <c r="BM131" t="n">
-        <v>0.6502477111911013</v>
+        <v>0.6502477111911014</v>
       </c>
       <c r="BN131" t="n">
         <v>1</v>
@@ -29699,7 +29699,7 @@
         <v>2592</v>
       </c>
       <c r="BM132" t="n">
-        <v>0.6588903588157287</v>
+        <v>0.6588903588157289</v>
       </c>
       <c r="BN132" t="n">
         <v>1</v>
@@ -29920,7 +29920,7 @@
         <v>2997</v>
       </c>
       <c r="BM133" t="n">
-        <v>0.6558177690486344</v>
+        <v>0.6558177690486343</v>
       </c>
       <c r="BN133" t="n">
         <v>1</v>
@@ -30141,7 +30141,7 @@
         <v>3078</v>
       </c>
       <c r="BM134" t="n">
-        <v>0.7193328946084493</v>
+        <v>0.7193328946084492</v>
       </c>
       <c r="BN134" t="n">
         <v>1</v>
@@ -31246,7 +31246,7 @@
         <v>3486</v>
       </c>
       <c r="BM139" t="n">
-        <v>0.7664126284368826</v>
+        <v>0.7664126284368825</v>
       </c>
       <c r="BN139" t="n">
         <v>1</v>
@@ -31909,7 +31909,7 @@
         <v>4565</v>
       </c>
       <c r="BM142" t="n">
-        <v>0.4996143784887053</v>
+        <v>0.4996143784887054</v>
       </c>
       <c r="BN142" t="n">
         <v>0</v>
@@ -33014,7 +33014,7 @@
         <v>4648</v>
       </c>
       <c r="BM147" t="n">
-        <v>0.5272443113753211</v>
+        <v>0.5272443113753212</v>
       </c>
       <c r="BN147" t="n">
         <v>1</v>
@@ -33677,7 +33677,7 @@
         <v>4316</v>
       </c>
       <c r="BM150" t="n">
-        <v>0.7981705418317234</v>
+        <v>0.7981705418317235</v>
       </c>
       <c r="BN150" t="n">
         <v>1</v>
@@ -34340,7 +34340,7 @@
         <v>5494</v>
       </c>
       <c r="BM153" t="n">
-        <v>0.4220848933832761</v>
+        <v>0.4220848933832762</v>
       </c>
       <c r="BN153" t="n">
         <v>0</v>
@@ -35003,7 +35003,7 @@
         <v>5248</v>
       </c>
       <c r="BM156" t="n">
-        <v>0.4079922880336398</v>
+        <v>0.4079922880336397</v>
       </c>
       <c r="BN156" t="n">
         <v>0</v>
@@ -35224,7 +35224,7 @@
         <v>6806</v>
       </c>
       <c r="BM157" t="n">
-        <v>0.3015849529801651</v>
+        <v>0.3015849529801652</v>
       </c>
       <c r="BN157" t="n">
         <v>0</v>
@@ -36329,7 +36329,7 @@
         <v>6806</v>
       </c>
       <c r="BM162" t="n">
-        <v>0.4351377200930648</v>
+        <v>0.4351377200930647</v>
       </c>
       <c r="BN162" t="n">
         <v>0</v>
@@ -36550,7 +36550,7 @@
         <v>6888</v>
       </c>
       <c r="BM163" t="n">
-        <v>0.5222516577503716</v>
+        <v>0.5222516577503717</v>
       </c>
       <c r="BN163" t="n">
         <v>1</v>
@@ -37655,7 +37655,7 @@
         <v>6205</v>
       </c>
       <c r="BM168" t="n">
-        <v>0.4719194555436784</v>
+        <v>0.4719194555436783</v>
       </c>
       <c r="BN168" t="n">
         <v>0</v>
@@ -38981,7 +38981,7 @@
         <v>4819</v>
       </c>
       <c r="BM174" t="n">
-        <v>0.5868649816170199</v>
+        <v>0.5868649816170198</v>
       </c>
       <c r="BN174" t="n">
         <v>1</v>
@@ -40749,7 +40749,7 @@
         <v>2968</v>
       </c>
       <c r="BM182" t="n">
-        <v>0.4688751570855096</v>
+        <v>0.4688751570855095</v>
       </c>
       <c r="BN182" t="n">
         <v>0</v>
@@ -40970,7 +40970,7 @@
         <v>3445</v>
       </c>
       <c r="BM183" t="n">
-        <v>0.5718939158978511</v>
+        <v>0.571893915897851</v>
       </c>
       <c r="BN183" t="n">
         <v>1</v>
@@ -41191,7 +41191,7 @@
         <v>4876</v>
       </c>
       <c r="BM184" t="n">
-        <v>0.29098509090994</v>
+        <v>0.2909850909099399</v>
       </c>
       <c r="BN184" t="n">
         <v>0</v>
@@ -41412,7 +41412,7 @@
         <v>5512</v>
       </c>
       <c r="BM185" t="n">
-        <v>0.2147137146066941</v>
+        <v>0.2147137146066942</v>
       </c>
       <c r="BN185" t="n">
         <v>0</v>
@@ -47379,7 +47379,7 @@
         <v>6800</v>
       </c>
       <c r="BM212" t="n">
-        <v>0.1853256785070618</v>
+        <v>0.1853256785070619</v>
       </c>
       <c r="BN212" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
*Correção de duplicação de ordem em caso de execuçao instantanea, tratado. *Correção ordem executada parcialmente, agora a função tenta até executar totalmente dentro do primeiro minuto, *Implemetado novos campos no treinamento do modelo
</commit_message>
<xml_diff>
--- a/Rodovias/modelos_rodovias/doutor_manoel_hyppolito_rego_km_83_caraguatatuba_sp_rf_regimes/predicoes_teste.xlsx
+++ b/Rodovias/modelos_rodovias/doutor_manoel_hyppolito_rego_km_83_caraguatatuba_sp_rf_regimes/predicoes_teste.xlsx
@@ -969,7 +969,7 @@
         <v>8964</v>
       </c>
       <c r="BM2" t="n">
-        <v>0.3131644635617931</v>
+        <v>0.3131644635617932</v>
       </c>
       <c r="BN2" t="n">
         <v>0</v>
@@ -2074,7 +2074,7 @@
         <v>9240</v>
       </c>
       <c r="BM7" t="n">
-        <v>0.3039589674521104</v>
+        <v>0.3039589674521105</v>
       </c>
       <c r="BN7" t="n">
         <v>0</v>
@@ -4505,7 +4505,7 @@
         <v>5481</v>
       </c>
       <c r="BM18" t="n">
-        <v>0.5098548213862929</v>
+        <v>0.509854821386293</v>
       </c>
       <c r="BN18" t="n">
         <v>1</v>
@@ -5610,7 +5610,7 @@
         <v>6474</v>
       </c>
       <c r="BM23" t="n">
-        <v>0.3191210761417623</v>
+        <v>0.3191210761417622</v>
       </c>
       <c r="BN23" t="n">
         <v>0</v>
@@ -8483,7 +8483,7 @@
         <v>6391</v>
       </c>
       <c r="BM36" t="n">
-        <v>0.3860785137198294</v>
+        <v>0.3860785137198293</v>
       </c>
       <c r="BN36" t="n">
         <v>0</v>
@@ -9367,7 +9367,7 @@
         <v>5280</v>
       </c>
       <c r="BM40" t="n">
-        <v>0.3870467616926194</v>
+        <v>0.3870467616926192</v>
       </c>
       <c r="BN40" t="n">
         <v>0</v>
@@ -9588,7 +9588,7 @@
         <v>3680</v>
       </c>
       <c r="BM41" t="n">
-        <v>0.5335224082541328</v>
+        <v>0.533522408254133</v>
       </c>
       <c r="BN41" t="n">
         <v>1</v>
@@ -10251,7 +10251,7 @@
         <v>4400</v>
       </c>
       <c r="BM44" t="n">
-        <v>0.6990215137655805</v>
+        <v>0.6990215137655804</v>
       </c>
       <c r="BN44" t="n">
         <v>1</v>
@@ -10472,7 +10472,7 @@
         <v>4400</v>
       </c>
       <c r="BM45" t="n">
-        <v>0.6883937679306908</v>
+        <v>0.6883937679306907</v>
       </c>
       <c r="BN45" t="n">
         <v>1</v>
@@ -10914,7 +10914,7 @@
         <v>4725</v>
       </c>
       <c r="BM47" t="n">
-        <v>0.5846708635149641</v>
+        <v>0.5846708635149643</v>
       </c>
       <c r="BN47" t="n">
         <v>1</v>
@@ -11798,7 +11798,7 @@
         <v>4800</v>
       </c>
       <c r="BM51" t="n">
-        <v>0.5706437627020653</v>
+        <v>0.5706437627020652</v>
       </c>
       <c r="BN51" t="n">
         <v>1</v>
@@ -12019,7 +12019,7 @@
         <v>4725</v>
       </c>
       <c r="BM52" t="n">
-        <v>0.6140954569271612</v>
+        <v>0.6140954569271613</v>
       </c>
       <c r="BN52" t="n">
         <v>1</v>
@@ -12461,7 +12461,7 @@
         <v>7700</v>
       </c>
       <c r="BM54" t="n">
-        <v>0.1150085075601559</v>
+        <v>0.115008507560156</v>
       </c>
       <c r="BN54" t="n">
         <v>0</v>
@@ -13787,7 +13787,7 @@
         <v>4140</v>
       </c>
       <c r="BM60" t="n">
-        <v>0.625463056641964</v>
+        <v>0.6254630566419639</v>
       </c>
       <c r="BN60" t="n">
         <v>1</v>
@@ -14450,7 +14450,7 @@
         <v>3243</v>
       </c>
       <c r="BM63" t="n">
-        <v>0.6382773049325777</v>
+        <v>0.6382773049325778</v>
       </c>
       <c r="BN63" t="n">
         <v>1</v>
@@ -15997,7 +15997,7 @@
         <v>3312</v>
       </c>
       <c r="BM70" t="n">
-        <v>0.65207572937864</v>
+        <v>0.6520757293786401</v>
       </c>
       <c r="BN70" t="n">
         <v>1</v>
@@ -17544,7 +17544,7 @@
         <v>8056</v>
       </c>
       <c r="BM77" t="n">
-        <v>0.1424768961083158</v>
+        <v>0.1424768961083157</v>
       </c>
       <c r="BN77" t="n">
         <v>0</v>
@@ -19091,7 +19091,7 @@
         <v>10320</v>
       </c>
       <c r="BM84" t="n">
-        <v>0.2712126107034817</v>
+        <v>0.2712126107034818</v>
       </c>
       <c r="BN84" t="n">
         <v>0</v>
@@ -19533,7 +19533,7 @@
         <v>6794</v>
       </c>
       <c r="BM86" t="n">
-        <v>0.5866083371239799</v>
+        <v>0.5866083371239801</v>
       </c>
       <c r="BN86" t="n">
         <v>1</v>
@@ -19754,7 +19754,7 @@
         <v>7568</v>
       </c>
       <c r="BM87" t="n">
-        <v>0.5039157593392207</v>
+        <v>0.5039157593392206</v>
       </c>
       <c r="BN87" t="n">
         <v>1</v>
@@ -21080,7 +21080,7 @@
         <v>7138</v>
       </c>
       <c r="BM93" t="n">
-        <v>0.4699803145743927</v>
+        <v>0.4699803145743928</v>
       </c>
       <c r="BN93" t="n">
         <v>0</v>
@@ -21301,7 +21301,7 @@
         <v>4644</v>
       </c>
       <c r="BM94" t="n">
-        <v>0.7555005771417855</v>
+        <v>0.7555005771417856</v>
       </c>
       <c r="BN94" t="n">
         <v>1</v>
@@ -21522,7 +21522,7 @@
         <v>4988</v>
       </c>
       <c r="BM95" t="n">
-        <v>0.5782682801356638</v>
+        <v>0.5782682801356639</v>
       </c>
       <c r="BN95" t="n">
         <v>1</v>
@@ -21964,7 +21964,7 @@
         <v>3864</v>
       </c>
       <c r="BM97" t="n">
-        <v>0.7153601247529701</v>
+        <v>0.7153601247529702</v>
       </c>
       <c r="BN97" t="n">
         <v>1</v>
@@ -24616,7 +24616,7 @@
         <v>4968</v>
       </c>
       <c r="BM109" t="n">
-        <v>0.6563706587057245</v>
+        <v>0.6563706587057244</v>
       </c>
       <c r="BN109" t="n">
         <v>1</v>
@@ -25058,7 +25058,7 @@
         <v>3990</v>
       </c>
       <c r="BM111" t="n">
-        <v>0.5965592438426691</v>
+        <v>0.5965592438426693</v>
       </c>
       <c r="BN111" t="n">
         <v>1</v>
@@ -25279,7 +25279,7 @@
         <v>5035</v>
       </c>
       <c r="BM112" t="n">
-        <v>0.6195030478644346</v>
+        <v>0.6195030478644344</v>
       </c>
       <c r="BN112" t="n">
         <v>1</v>
@@ -27710,7 +27710,7 @@
         <v>7695</v>
       </c>
       <c r="BM123" t="n">
-        <v>0.2960635545210544</v>
+        <v>0.2960635545210545</v>
       </c>
       <c r="BN123" t="n">
         <v>0</v>
@@ -28373,7 +28373,7 @@
         <v>2125</v>
       </c>
       <c r="BM126" t="n">
-        <v>0.721496108945355</v>
+        <v>0.7214961089453551</v>
       </c>
       <c r="BN126" t="n">
         <v>1</v>
@@ -29699,7 +29699,7 @@
         <v>2592</v>
       </c>
       <c r="BM132" t="n">
-        <v>0.6588903588157289</v>
+        <v>0.6588903588157287</v>
       </c>
       <c r="BN132" t="n">
         <v>1</v>
@@ -29920,7 +29920,7 @@
         <v>2997</v>
       </c>
       <c r="BM133" t="n">
-        <v>0.6558177690486343</v>
+        <v>0.6558177690486344</v>
       </c>
       <c r="BN133" t="n">
         <v>1</v>
@@ -31246,7 +31246,7 @@
         <v>3486</v>
       </c>
       <c r="BM139" t="n">
-        <v>0.7664126284368825</v>
+        <v>0.7664126284368826</v>
       </c>
       <c r="BN139" t="n">
         <v>1</v>
@@ -31467,7 +31467,7 @@
         <v>3901</v>
       </c>
       <c r="BM140" t="n">
-        <v>0.7136187398919878</v>
+        <v>0.7136187398919875</v>
       </c>
       <c r="BN140" t="n">
         <v>1</v>
@@ -31909,7 +31909,7 @@
         <v>4565</v>
       </c>
       <c r="BM142" t="n">
-        <v>0.4996143784887054</v>
+        <v>0.4996143784887053</v>
       </c>
       <c r="BN142" t="n">
         <v>0</v>
@@ -32130,7 +32130,7 @@
         <v>4233</v>
       </c>
       <c r="BM143" t="n">
-        <v>0.7190469794572577</v>
+        <v>0.7190469794572576</v>
       </c>
       <c r="BN143" t="n">
         <v>1</v>
@@ -33014,7 +33014,7 @@
         <v>4648</v>
       </c>
       <c r="BM147" t="n">
-        <v>0.5272443113753212</v>
+        <v>0.5272443113753211</v>
       </c>
       <c r="BN147" t="n">
         <v>1</v>
@@ -34340,7 +34340,7 @@
         <v>5494</v>
       </c>
       <c r="BM153" t="n">
-        <v>0.4220848933832762</v>
+        <v>0.4220848933832761</v>
       </c>
       <c r="BN153" t="n">
         <v>0</v>
@@ -36550,7 +36550,7 @@
         <v>6888</v>
       </c>
       <c r="BM163" t="n">
-        <v>0.5222516577503717</v>
+        <v>0.5222516577503716</v>
       </c>
       <c r="BN163" t="n">
         <v>1</v>
@@ -36771,7 +36771,7 @@
         <v>6068</v>
       </c>
       <c r="BM164" t="n">
-        <v>0.4817014105705811</v>
+        <v>0.481701410570581</v>
       </c>
       <c r="BN164" t="n">
         <v>0</v>
@@ -36992,7 +36992,7 @@
         <v>5548</v>
       </c>
       <c r="BM165" t="n">
-        <v>0.4375107596113822</v>
+        <v>0.4375107596113821</v>
       </c>
       <c r="BN165" t="n">
         <v>0</v>
@@ -38981,7 +38981,7 @@
         <v>4819</v>
       </c>
       <c r="BM174" t="n">
-        <v>0.5868649816170198</v>
+        <v>0.5868649816170197</v>
       </c>
       <c r="BN174" t="n">
         <v>1</v>
@@ -39202,7 +39202,7 @@
         <v>4392</v>
       </c>
       <c r="BM175" t="n">
-        <v>0.507619762437946</v>
+        <v>0.5076197624379459</v>
       </c>
       <c r="BN175" t="n">
         <v>1</v>
@@ -40749,7 +40749,7 @@
         <v>2968</v>
       </c>
       <c r="BM182" t="n">
-        <v>0.4688751570855095</v>
+        <v>0.4688751570855096</v>
       </c>
       <c r="BN182" t="n">
         <v>0</v>
@@ -40970,7 +40970,7 @@
         <v>3445</v>
       </c>
       <c r="BM183" t="n">
-        <v>0.571893915897851</v>
+        <v>0.5718939158978511</v>
       </c>
       <c r="BN183" t="n">
         <v>1</v>
@@ -41191,7 +41191,7 @@
         <v>4876</v>
       </c>
       <c r="BM184" t="n">
-        <v>0.2909850909099399</v>
+        <v>0.29098509090994</v>
       </c>
       <c r="BN184" t="n">
         <v>0</v>
@@ -41854,7 +41854,7 @@
         <v>2652</v>
       </c>
       <c r="BM187" t="n">
-        <v>0.5759554423406754</v>
+        <v>0.5759554423406752</v>
       </c>
       <c r="BN187" t="n">
         <v>1</v>
@@ -42075,7 +42075,7 @@
         <v>5151</v>
       </c>
       <c r="BM188" t="n">
-        <v>0.211447158560292</v>
+        <v>0.2114471585602921</v>
       </c>
       <c r="BN188" t="n">
         <v>0</v>
@@ -42517,7 +42517,7 @@
         <v>2907</v>
       </c>
       <c r="BM190" t="n">
-        <v>0.5954282609559413</v>
+        <v>0.5954282609559414</v>
       </c>
       <c r="BN190" t="n">
         <v>1</v>
@@ -44285,7 +44285,7 @@
         <v>4292</v>
       </c>
       <c r="BM198" t="n">
-        <v>0.3574922586604519</v>
+        <v>0.357492258660452</v>
       </c>
       <c r="BN198" t="n">
         <v>0</v>
@@ -45169,7 +45169,7 @@
         <v>3283</v>
       </c>
       <c r="BM202" t="n">
-        <v>0.5601337137276169</v>
+        <v>0.5601337137276168</v>
       </c>
       <c r="BN202" t="n">
         <v>1</v>
@@ -45390,7 +45390,7 @@
         <v>3953</v>
       </c>
       <c r="BM203" t="n">
-        <v>0.6017793605665199</v>
+        <v>0.60177936056652</v>
       </c>
       <c r="BN203" t="n">
         <v>1</v>
@@ -47379,7 +47379,7 @@
         <v>6800</v>
       </c>
       <c r="BM212" t="n">
-        <v>0.1853256785070619</v>
+        <v>0.1853256785070618</v>
       </c>
       <c r="BN212" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Versão com implementação de dados de passagem
</commit_message>
<xml_diff>
--- a/Rodovias/modelos_rodovias/doutor_manoel_hyppolito_rego_km_83_caraguatatuba_sp_rf_regimes/predicoes_teste.xlsx
+++ b/Rodovias/modelos_rodovias/doutor_manoel_hyppolito_rego_km_83_caraguatatuba_sp_rf_regimes/predicoes_teste.xlsx
@@ -3343,7 +3343,7 @@
         <v>5456</v>
       </c>
       <c r="BX11" t="n">
-        <v>0.6551449417191502</v>
+        <v>0.6551449417191503</v>
       </c>
       <c r="BY11" t="n">
         <v>1</v>
@@ -4867,7 +4867,7 @@
         <v>5394</v>
       </c>
       <c r="BX17" t="n">
-        <v>0.5371508432747726</v>
+        <v>0.5371508432747727</v>
       </c>
       <c r="BY17" t="n">
         <v>1</v>
@@ -6645,7 +6645,7 @@
         <v>4543</v>
       </c>
       <c r="BX24" t="n">
-        <v>0.3908963861346712</v>
+        <v>0.3908963861346711</v>
       </c>
       <c r="BY24" t="n">
         <v>0</v>
@@ -8931,7 +8931,7 @@
         <v>7238</v>
       </c>
       <c r="BX33" t="n">
-        <v>0.408175734543651</v>
+        <v>0.4081757345436511</v>
       </c>
       <c r="BY33" t="n">
         <v>0</v>
@@ -9947,7 +9947,7 @@
         <v>7777</v>
       </c>
       <c r="BX37" t="n">
-        <v>0.4102645031410284</v>
+        <v>0.4102645031410283</v>
       </c>
       <c r="BY37" t="n">
         <v>0</v>
@@ -10201,7 +10201,7 @@
         <v>7315</v>
       </c>
       <c r="BX38" t="n">
-        <v>0.544419177867696</v>
+        <v>0.5444191778676959</v>
       </c>
       <c r="BY38" t="n">
         <v>1</v>
@@ -12487,7 +12487,7 @@
         <v>4725</v>
       </c>
       <c r="BX47" t="n">
-        <v>0.4426335618651556</v>
+        <v>0.4426335618651557</v>
       </c>
       <c r="BY47" t="n">
         <v>0</v>
@@ -16551,7 +16551,7 @@
         <v>3243</v>
       </c>
       <c r="BX63" t="n">
-        <v>0.6119483150084994</v>
+        <v>0.6119483150084993</v>
       </c>
       <c r="BY63" t="n">
         <v>1</v>
@@ -21885,7 +21885,7 @@
         <v>10320</v>
       </c>
       <c r="BX84" t="n">
-        <v>0.1715726485878392</v>
+        <v>0.1715726485878393</v>
       </c>
       <c r="BY84" t="n">
         <v>0</v>
@@ -23917,7 +23917,7 @@
         <v>9288</v>
       </c>
       <c r="BX92" t="n">
-        <v>0.1758501503897599</v>
+        <v>0.17585015038976</v>
       </c>
       <c r="BY92" t="n">
         <v>0</v>
@@ -24933,7 +24933,7 @@
         <v>4988</v>
       </c>
       <c r="BX96" t="n">
-        <v>0.5553814390459946</v>
+        <v>0.5553814390459945</v>
       </c>
       <c r="BY96" t="n">
         <v>1</v>
@@ -25441,7 +25441,7 @@
         <v>4968</v>
       </c>
       <c r="BX98" t="n">
-        <v>0.5163971684363751</v>
+        <v>0.5163971684363752</v>
       </c>
       <c r="BY98" t="n">
         <v>1</v>
@@ -27219,7 +27219,7 @@
         <v>7820</v>
       </c>
       <c r="BX105" t="n">
-        <v>0.515361428200263</v>
+        <v>0.5153614282002629</v>
       </c>
       <c r="BY105" t="n">
         <v>1</v>
@@ -28235,7 +28235,7 @@
         <v>4968</v>
       </c>
       <c r="BX109" t="n">
-        <v>0.6570599793418411</v>
+        <v>0.6570599793418412</v>
       </c>
       <c r="BY109" t="n">
         <v>1</v>
@@ -28743,7 +28743,7 @@
         <v>3990</v>
       </c>
       <c r="BX111" t="n">
-        <v>0.6330796745329145</v>
+        <v>0.6330796745329144</v>
       </c>
       <c r="BY111" t="n">
         <v>1</v>
@@ -29251,7 +29251,7 @@
         <v>7220</v>
       </c>
       <c r="BX113" t="n">
-        <v>0.5108141635811992</v>
+        <v>0.5108141635811991</v>
       </c>
       <c r="BY113" t="n">
         <v>1</v>
@@ -29505,7 +29505,7 @@
         <v>8455</v>
       </c>
       <c r="BX114" t="n">
-        <v>0.4029472278728774</v>
+        <v>0.4029472278728773</v>
       </c>
       <c r="BY114" t="n">
         <v>0</v>
@@ -32045,7 +32045,7 @@
         <v>1530</v>
       </c>
       <c r="BX124" t="n">
-        <v>0.779342774996248</v>
+        <v>0.7793427749962479</v>
       </c>
       <c r="BY124" t="n">
         <v>1</v>
@@ -32553,7 +32553,7 @@
         <v>2125</v>
       </c>
       <c r="BX126" t="n">
-        <v>0.6317612304813069</v>
+        <v>0.6317612304813072</v>
       </c>
       <c r="BY126" t="n">
         <v>1</v>
@@ -33315,7 +33315,7 @@
         <v>1944</v>
       </c>
       <c r="BX129" t="n">
-        <v>0.728777473551798</v>
+        <v>0.7287774735517979</v>
       </c>
       <c r="BY129" t="n">
         <v>1</v>
@@ -34077,7 +34077,7 @@
         <v>2592</v>
       </c>
       <c r="BX132" t="n">
-        <v>0.6800218350143912</v>
+        <v>0.680021835014391</v>
       </c>
       <c r="BY132" t="n">
         <v>1</v>
@@ -34585,7 +34585,7 @@
         <v>3078</v>
       </c>
       <c r="BX134" t="n">
-        <v>0.7248794271226551</v>
+        <v>0.724879427122655</v>
       </c>
       <c r="BY134" t="n">
         <v>1</v>
@@ -35093,7 +35093,7 @@
         <v>3564</v>
       </c>
       <c r="BX136" t="n">
-        <v>0.6965884952795783</v>
+        <v>0.6965884952795781</v>
       </c>
       <c r="BY136" t="n">
         <v>1</v>
@@ -35347,7 +35347,7 @@
         <v>4050</v>
       </c>
       <c r="BX137" t="n">
-        <v>0.7417192568432881</v>
+        <v>0.7417192568432882</v>
       </c>
       <c r="BY137" t="n">
         <v>1</v>
@@ -36109,7 +36109,7 @@
         <v>3901</v>
       </c>
       <c r="BX140" t="n">
-        <v>0.7331055699033117</v>
+        <v>0.7331055699033118</v>
       </c>
       <c r="BY140" t="n">
         <v>1</v>
@@ -37379,7 +37379,7 @@
         <v>2573</v>
       </c>
       <c r="BX145" t="n">
-        <v>0.8128045905694685</v>
+        <v>0.8128045905694684</v>
       </c>
       <c r="BY145" t="n">
         <v>1</v>
@@ -37887,7 +37887,7 @@
         <v>4648</v>
       </c>
       <c r="BX147" t="n">
-        <v>0.6621433891900796</v>
+        <v>0.6621433891900795</v>
       </c>
       <c r="BY147" t="n">
         <v>1</v>
@@ -38141,7 +38141,7 @@
         <v>4814</v>
       </c>
       <c r="BX148" t="n">
-        <v>0.6192790010578235</v>
+        <v>0.6192790010578236</v>
       </c>
       <c r="BY148" t="n">
         <v>1</v>
@@ -41189,7 +41189,7 @@
         <v>3936</v>
       </c>
       <c r="BX160" t="n">
-        <v>0.7475389244430078</v>
+        <v>0.747538924443008</v>
       </c>
       <c r="BY160" t="n">
         <v>1</v>
@@ -42205,7 +42205,7 @@
         <v>6068</v>
       </c>
       <c r="BX164" t="n">
-        <v>0.6170462157293389</v>
+        <v>0.617046215729339</v>
       </c>
       <c r="BY164" t="n">
         <v>1</v>
@@ -46015,7 +46015,7 @@
         <v>3021</v>
       </c>
       <c r="BX179" t="n">
-        <v>0.6883437290317989</v>
+        <v>0.688343729031799</v>
       </c>
       <c r="BY179" t="n">
         <v>1</v>
@@ -47285,7 +47285,7 @@
         <v>4876</v>
       </c>
       <c r="BX184" t="n">
-        <v>0.2909967273387253</v>
+        <v>0.2909967273387252</v>
       </c>
       <c r="BY184" t="n">
         <v>0</v>
@@ -49317,7 +49317,7 @@
         <v>3392</v>
       </c>
       <c r="BX192" t="n">
-        <v>0.5262771288720808</v>
+        <v>0.5262771288720809</v>
       </c>
       <c r="BY192" t="n">
         <v>1</v>
@@ -49571,7 +49571,7 @@
         <v>2756</v>
       </c>
       <c r="BX193" t="n">
-        <v>0.5699454345073812</v>
+        <v>0.5699454345073813</v>
       </c>
       <c r="BY193" t="n">
         <v>1</v>
@@ -53635,7 +53635,7 @@
         <v>7772</v>
       </c>
       <c r="BX209" t="n">
-        <v>0.1834498514908788</v>
+        <v>0.1834498514908787</v>
       </c>
       <c r="BY209" t="n">
         <v>0</v>
@@ -55667,7 +55667,7 @@
         <v>7081</v>
       </c>
       <c r="BX217" t="n">
-        <v>0.3822589180887734</v>
+        <v>0.3822589180887733</v>
       </c>
       <c r="BY217" t="n">
         <v>0</v>
@@ -56683,7 +56683,7 @@
         <v>1680</v>
       </c>
       <c r="BX221" t="n">
-        <v>0.3911217299508298</v>
+        <v>0.3911217299508297</v>
       </c>
       <c r="BY221" t="n">
         <v>0</v>

</xml_diff>